<commit_message>
Changes made in Del-1: Rapport
</commit_message>
<xml_diff>
--- a/Del_1-Rapport/Jämförelsetabell_CI_CD_CD.xlsx
+++ b/Del_1-Rapport/Jämförelsetabell_CI_CD_CD.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Studies\Testautomation_CI_CD\InlämningsUppgift_TA\Del_1-Rapport\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39B2B3CF-ED9A-4D97-9873-80A1669D5E99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4386249B-5745-45B0-A2CF-CA94B25FC303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{07C83AA5-0C0D-4C6E-A5D3-626AFFE9DFDD}"/>
+    <workbookView xWindow="-28020" yWindow="780" windowWidth="21600" windowHeight="11235" xr2:uid="{07C83AA5-0C0D-4C6E-A5D3-626AFFE9DFDD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -125,9 +125,6 @@
     <t xml:space="preserve"> Nej ( Push elle Pull request är manuellt)</t>
   </si>
   <si>
-    <t xml:space="preserve"> Full regression, Danary, A/B</t>
-  </si>
-  <si>
     <t>Acceptanstester i staging</t>
   </si>
   <si>
@@ -135,6 +132,9 @@
   </si>
   <si>
     <t xml:space="preserve">Jämförelsetabell CI vs Continuous Delivery vs Continuous Deployment </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Full regression</t>
   </si>
 </sst>
 </file>
@@ -573,7 +573,7 @@
   <sheetData>
     <row r="1" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B1" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
@@ -649,10 +649,10 @@
         <v>16</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="2:5" ht="42" customHeight="1" x14ac:dyDescent="0.35">
@@ -666,7 +666,7 @@
         <v>19</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="2:5" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>